<commit_message>
gui cleanup, download button
</commit_message>
<xml_diff>
--- a/Validation Study/Final_Validity.xlsx
+++ b/Validation Study/Final_Validity.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Anthony\Desktop\peak_detector\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Anthony\Desktop\peak_detector\Validation Study\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2579512E-8B9B-4F12-B37C-72B0AB4E83FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44F95FE1-9F3F-4ECA-A392-5FBEBBE69232}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8DC5E736-AF77-4E0E-91F2-31C73D6083CB}"/>
   </bookViews>
@@ -161,7 +161,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -174,6 +174,14 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -973,92 +981,92 @@
         <v>449.29232329878897</v>
       </c>
     </row>
-    <row r="6" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A6">
+    <row r="6" spans="1:29" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="6">
         <v>5</v>
       </c>
-      <c r="B6" s="1">
+      <c r="B6" s="7">
         <v>304</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6" s="7">
         <v>304</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="6">
         <v>61.3024236037934</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="7">
         <v>61.3</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="6">
         <v>978.75412541254104</v>
       </c>
-      <c r="G6">
+      <c r="G6" s="6">
         <v>978.75412541254104</v>
       </c>
-      <c r="H6">
+      <c r="H6" s="6">
         <v>65.127099989499101</v>
       </c>
-      <c r="I6">
+      <c r="I6" s="6">
         <v>65.127099989499101</v>
       </c>
-      <c r="J6">
+      <c r="J6" s="6">
         <v>43.894389438943797</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="7">
         <v>43.75</v>
       </c>
-      <c r="L6">
+      <c r="L6" s="6">
         <v>46.710128260444201</v>
       </c>
-      <c r="M6">
+      <c r="M6" s="6">
         <v>46.632985138829298</v>
       </c>
-      <c r="N6">
+      <c r="N6" s="6">
         <v>46.128248640312599</v>
       </c>
-      <c r="O6">
+      <c r="O6" s="6">
         <v>27.337018772755499</v>
       </c>
-      <c r="P6">
+      <c r="P6" s="6">
         <v>47.318160592401703</v>
       </c>
-      <c r="Q6">
+      <c r="Q6" s="6">
         <v>60.016314536420602</v>
       </c>
-      <c r="R6" s="1">
+      <c r="R6" s="7">
         <v>0.97485295418942897</v>
       </c>
-      <c r="S6">
+      <c r="S6" s="6">
         <v>0.45549312689245702</v>
       </c>
-      <c r="T6">
+      <c r="T6" s="6">
         <v>0.74966279061415397</v>
       </c>
-      <c r="U6">
+      <c r="U6" s="6">
         <v>0.69151115577418598</v>
       </c>
-      <c r="V6">
+      <c r="V6" s="6">
         <v>0.42874107393758498</v>
       </c>
-      <c r="W6">
+      <c r="W6" s="6">
         <v>0.408812648627013</v>
       </c>
-      <c r="X6">
+      <c r="X6" s="6">
         <v>0.57125892606241402</v>
       </c>
-      <c r="Y6">
+      <c r="Y6" s="6">
         <v>0.59118735137298595</v>
       </c>
-      <c r="Z6">
+      <c r="Z6" s="6">
         <v>634.36549424860095</v>
       </c>
-      <c r="AA6" s="5">
+      <c r="AA6" s="8">
         <v>588.78634979060303</v>
       </c>
-      <c r="AB6" s="2">
+      <c r="AB6" s="9">
         <v>846.20112161216196</v>
       </c>
-      <c r="AC6" s="5">
+      <c r="AC6" s="8">
         <v>851.44880870565703</v>
       </c>
     </row>

</xml_diff>